<commit_message>
se cargan archivos y sql view de encuestas fatlab 06_05_2026
</commit_message>
<xml_diff>
--- a/DataSphere/Encuestas Satisfaccion/Check areas realizadas Script.xlsx
+++ b/DataSphere/Encuestas Satisfaccion/Check areas realizadas Script.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\degonzalez\Documents\2026\Backup_2026\DataSphere\Encuestas Satisfaccion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Favorites\Daniel\Backup_2026\DataSphere\Encuestas Satisfaccion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DCB5340-9918-47AD-8662-25866BE60A9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D4F9F18-2F9E-4054-8C67-5E491F54450C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{7AC92B9D-D867-42DF-A351-213DC04F481B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7AC92B9D-D867-42DF-A351-213DC04F481B}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="24">
   <si>
     <t xml:space="preserve">Area </t>
   </si>
@@ -111,6 +111,9 @@
   </si>
   <si>
     <t>item</t>
+  </si>
+  <si>
+    <t>en proceso</t>
   </si>
 </sst>
 </file>
@@ -483,12 +486,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E32B2A4E-C96F-42B7-B01F-CBD69B9FB44F}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="52.5703125" customWidth="1"/>
+    <col min="2" max="2" width="52.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>22</v>
       </c>
@@ -499,7 +502,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -510,55 +513,73 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -566,7 +587,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -574,7 +595,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -582,7 +603,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -590,7 +611,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -598,7 +619,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -606,7 +627,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -614,7 +635,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
@@ -622,7 +643,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -630,7 +651,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
@@ -638,7 +659,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
@@ -646,7 +667,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>

</xml_diff>